<commit_message>
Artist Apis done halfway
</commit_message>
<xml_diff>
--- a/other/Streaming Music Platform API doc.xlsx
+++ b/other/Streaming Music Platform API doc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://husteduvn-my.sharepoint.com/personal/nam_pt207622_sis_hust_edu_vn/Documents/20242 - Final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nampt\Study\Music-Streaming-Platform-With-Audio-Search-Feature\other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="342" documentId="8_{590DE904-961F-43A0-989F-38C3CAB7648B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{689C0293-AF3B-4EB0-A354-833CB409D2FC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEE193F-E48E-4205-B973-2FFA6083DEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-3495" windowWidth="29040" windowHeight="15720" xr2:uid="{ED7FCC31-D23E-4CB2-901E-5DB0C03D8054}"/>
+    <workbookView xWindow="19080" yWindow="3660" windowWidth="20730" windowHeight="11040" xr2:uid="{ED7FCC31-D23E-4CB2-901E-5DB0C03D8054}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="112">
   <si>
     <t>User</t>
   </si>
@@ -188,16 +188,10 @@
     <t>Get tracks information</t>
   </si>
   <si>
-    <t>Stream track</t>
-  </si>
-  <si>
     <t xml:space="preserve">name, duration, artistId, albumId, coverUrl, cdnUrl </t>
   </si>
   <si>
     <t>name, artistId, albumId, coverUrl</t>
-  </si>
-  <si>
-    <t>/tracks/info/{id}</t>
   </si>
   <si>
     <t>/artists/{id}</t>
@@ -535,10 +529,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -858,16 +848,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45645413-E01D-4921-8D2A-99935D3359A4}">
-  <dimension ref="A2:H150"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A2:H149"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" customWidth="1"/>
-    <col min="2" max="4" width="22.6328125" customWidth="1"/>
-    <col min="5" max="5" width="26.6328125" customWidth="1"/>
-    <col min="6" max="8" width="22.6328125" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="2" max="4" width="22.5703125" customWidth="1"/>
+    <col min="5" max="5" width="26.5703125" customWidth="1"/>
+    <col min="6" max="8" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -890,10 +880,10 @@
         <v>5</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" s="5" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="5" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>33</v>
       </c>
@@ -913,13 +903,13 @@
         <v>39</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="5" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="5" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>12</v>
@@ -935,103 +925,103 @@
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="5" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="5" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>39</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="5" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" s="5" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="5" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="5" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="5" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>0</v>
       </c>
@@ -1054,10 +1044,10 @@
         <v>11</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
@@ -1078,10 +1068,10 @@
         <v>16</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="1" t="s">
         <v>18</v>
@@ -1103,7 +1093,7 @@
       </c>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="1" t="s">
         <v>8</v>
@@ -1125,7 +1115,7 @@
       </c>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="1" t="s">
         <v>8</v>
@@ -1145,9 +1135,11 @@
       <c r="G13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H13" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="1" t="s">
         <v>17</v>
@@ -1167,9 +1159,11 @@
       <c r="G14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H14" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="1" t="s">
         <v>17</v>
@@ -1189,9 +1183,11 @@
       <c r="G15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H15" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="1" t="s">
         <v>17</v>
@@ -1211,9 +1207,11 @@
       <c r="G16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="H16" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>40</v>
       </c>
@@ -1227,17 +1225,19 @@
         <v>42</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
       <c r="B18" s="1" t="s">
         <v>43</v>
@@ -1249,17 +1249,19 @@
         <v>46</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="12"/>
       <c r="B19" s="1" t="s">
         <v>18</v>
@@ -1271,15 +1273,17 @@
         <v>45</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
       <c r="B20" s="1" t="s">
         <v>17</v>
@@ -1291,55 +1295,61 @@
         <v>48</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H20" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
       <c r="B21" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H21" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
       <c r="B22" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H22" s="4"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H22" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
       <c r="B23" s="1" t="s">
         <v>17</v>
@@ -1348,137 +1358,151 @@
         <v>44</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="12"/>
+      <c r="H23" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>81</v>
+      </c>
       <c r="B24" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F24" s="1"/>
+        <v>59</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="G24" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A25" s="12" t="s">
-        <v>83</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
       <c r="B25" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H25" s="4"/>
-    </row>
-    <row r="26" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>66</v>
+        <v>53</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H26" s="4"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
       <c r="B27" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F27" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
       <c r="B28" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>57</v>
+      <c r="E28" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="H28" s="4"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="12"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="B29" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>10</v>
@@ -1487,181 +1511,179 @@
         <v>10</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="H29" s="4"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="12" t="s">
-        <v>84</v>
-      </c>
+    <row r="30" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="12"/>
       <c r="B30" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F30" s="3" t="s">
-        <v>10</v>
+      <c r="F30" s="7" t="s">
+        <v>65</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H30" s="4"/>
     </row>
-    <row r="31" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
       <c r="B31" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>75</v>
+        <v>12</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>66</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F31" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="E31" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="G31" s="1" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="H31" s="4"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="12"/>
       <c r="B32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="E32" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="12"/>
       <c r="B33" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E33" s="1" t="s">
         <v>72</v>
       </c>
+      <c r="E33" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="F33" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H33" s="4"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" s="12"/>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>84</v>
+      </c>
       <c r="B34" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="12" t="s">
-        <v>86</v>
-      </c>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="12"/>
       <c r="B35" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H35" s="4"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>10</v>
+        <v>96</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>93</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H36" s="4"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>95</v>
+        <v>88</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>10</v>
@@ -1671,19 +1693,19 @@
       </c>
       <c r="H37" s="4"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>10</v>
@@ -1693,19 +1715,19 @@
       </c>
       <c r="H38" s="4"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="12"/>
       <c r="B39" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>10</v>
@@ -1715,19 +1737,19 @@
       </c>
       <c r="H39" s="4"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="12"/>
       <c r="B40" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>10</v>
@@ -1737,29 +1759,16 @@
       </c>
       <c r="H40" s="4"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41" s="12"/>
-      <c r="B41" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H41" s="4"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -1768,7 +1777,7 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
@@ -1777,7 +1786,7 @@
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
@@ -1786,7 +1795,7 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
@@ -1795,7 +1804,7 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -1804,7 +1813,7 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
@@ -1813,7 +1822,7 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
@@ -1822,7 +1831,7 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
@@ -1831,7 +1840,7 @@
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
@@ -1840,7 +1849,7 @@
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
@@ -1849,7 +1858,7 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
       <c r="D52" s="1"/>
@@ -1858,7 +1867,7 @@
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -1867,7 +1876,7 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
       <c r="D54" s="1"/>
@@ -1876,7 +1885,7 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
@@ -1885,7 +1894,7 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
@@ -1894,7 +1903,7 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
@@ -1903,7 +1912,7 @@
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
@@ -1912,16 +1921,15 @@
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-    </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
@@ -1929,7 +1937,7 @@
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
     </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -1937,7 +1945,7 @@
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
@@ -1945,7 +1953,7 @@
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
@@ -1953,7 +1961,7 @@
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
     </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
@@ -1961,7 +1969,7 @@
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
@@ -1969,7 +1977,7 @@
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
@@ -1977,7 +1985,7 @@
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
@@ -1985,7 +1993,7 @@
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
@@ -1993,7 +2001,7 @@
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -2001,7 +2009,7 @@
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
@@ -2009,7 +2017,7 @@
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
@@ -2017,7 +2025,7 @@
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
@@ -2025,7 +2033,7 @@
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
       <c r="D73" s="1"/>
@@ -2033,7 +2041,7 @@
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -2041,7 +2049,7 @@
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
@@ -2049,7 +2057,7 @@
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
@@ -2057,7 +2065,7 @@
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
@@ -2065,7 +2073,7 @@
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
@@ -2073,7 +2081,7 @@
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
@@ -2081,7 +2089,7 @@
       <c r="F79" s="1"/>
       <c r="G79" s="1"/>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
@@ -2089,7 +2097,7 @@
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
@@ -2097,7 +2105,7 @@
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
@@ -2105,7 +2113,7 @@
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
       <c r="D83" s="1"/>
@@ -2113,7 +2121,7 @@
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
       <c r="D84" s="1"/>
@@ -2121,7 +2129,7 @@
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
@@ -2129,7 +2137,7 @@
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
       <c r="D86" s="1"/>
@@ -2137,7 +2145,7 @@
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
       <c r="D87" s="1"/>
@@ -2145,7 +2153,7 @@
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
       <c r="D88" s="1"/>
@@ -2153,7 +2161,7 @@
       <c r="F88" s="1"/>
       <c r="G88" s="1"/>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
       <c r="D89" s="1"/>
@@ -2161,7 +2169,7 @@
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
@@ -2169,7 +2177,7 @@
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
       <c r="D91" s="1"/>
@@ -2177,7 +2185,7 @@
       <c r="F91" s="1"/>
       <c r="G91" s="1"/>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
       <c r="D92" s="1"/>
@@ -2185,7 +2193,7 @@
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
       <c r="D93" s="1"/>
@@ -2193,7 +2201,7 @@
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
       <c r="D94" s="1"/>
@@ -2201,7 +2209,7 @@
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
       <c r="D95" s="1"/>
@@ -2209,7 +2217,7 @@
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
       <c r="D96" s="1"/>
@@ -2217,7 +2225,7 @@
       <c r="F96" s="1"/>
       <c r="G96" s="1"/>
     </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
       <c r="D97" s="1"/>
@@ -2225,7 +2233,7 @@
       <c r="F97" s="1"/>
       <c r="G97" s="1"/>
     </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
@@ -2233,7 +2241,7 @@
       <c r="F98" s="1"/>
       <c r="G98" s="1"/>
     </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
@@ -2241,7 +2249,7 @@
       <c r="F99" s="1"/>
       <c r="G99" s="1"/>
     </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
       <c r="D100" s="1"/>
@@ -2249,7 +2257,7 @@
       <c r="F100" s="1"/>
       <c r="G100" s="1"/>
     </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
       <c r="D101" s="1"/>
@@ -2257,7 +2265,7 @@
       <c r="F101" s="1"/>
       <c r="G101" s="1"/>
     </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
       <c r="D102" s="1"/>
@@ -2265,7 +2273,7 @@
       <c r="F102" s="1"/>
       <c r="G102" s="1"/>
     </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
       <c r="D103" s="1"/>
@@ -2273,7 +2281,7 @@
       <c r="F103" s="1"/>
       <c r="G103" s="1"/>
     </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
       <c r="D104" s="1"/>
@@ -2281,7 +2289,7 @@
       <c r="F104" s="1"/>
       <c r="G104" s="1"/>
     </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
       <c r="D105" s="1"/>
@@ -2289,7 +2297,7 @@
       <c r="F105" s="1"/>
       <c r="G105" s="1"/>
     </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
       <c r="D106" s="1"/>
@@ -2297,7 +2305,7 @@
       <c r="F106" s="1"/>
       <c r="G106" s="1"/>
     </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
       <c r="D107" s="1"/>
@@ -2305,7 +2313,7 @@
       <c r="F107" s="1"/>
       <c r="G107" s="1"/>
     </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
       <c r="D108" s="1"/>
@@ -2313,7 +2321,7 @@
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
     </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
       <c r="D109" s="1"/>
@@ -2321,7 +2329,7 @@
       <c r="F109" s="1"/>
       <c r="G109" s="1"/>
     </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
       <c r="D110" s="1"/>
@@ -2329,7 +2337,7 @@
       <c r="F110" s="1"/>
       <c r="G110" s="1"/>
     </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
       <c r="D111" s="1"/>
@@ -2337,7 +2345,7 @@
       <c r="F111" s="1"/>
       <c r="G111" s="1"/>
     </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
       <c r="D112" s="1"/>
@@ -2345,7 +2353,7 @@
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
       <c r="D113" s="1"/>
@@ -2353,7 +2361,7 @@
       <c r="F113" s="1"/>
       <c r="G113" s="1"/>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
       <c r="D114" s="1"/>
@@ -2361,7 +2369,7 @@
       <c r="F114" s="1"/>
       <c r="G114" s="1"/>
     </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
       <c r="D115" s="1"/>
@@ -2369,7 +2377,7 @@
       <c r="F115" s="1"/>
       <c r="G115" s="1"/>
     </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
       <c r="D116" s="1"/>
@@ -2377,7 +2385,7 @@
       <c r="F116" s="1"/>
       <c r="G116" s="1"/>
     </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
       <c r="D117" s="1"/>
@@ -2385,7 +2393,7 @@
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
     </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
       <c r="D118" s="1"/>
@@ -2393,7 +2401,7 @@
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
     </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
       <c r="D119" s="1"/>
@@ -2401,7 +2409,7 @@
       <c r="F119" s="1"/>
       <c r="G119" s="1"/>
     </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
       <c r="D120" s="1"/>
@@ -2409,7 +2417,7 @@
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
     </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
       <c r="D121" s="1"/>
@@ -2417,7 +2425,7 @@
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
     </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
       <c r="D122" s="1"/>
@@ -2425,7 +2433,7 @@
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
     </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
       <c r="D123" s="1"/>
@@ -2433,7 +2441,7 @@
       <c r="F123" s="1"/>
       <c r="G123" s="1"/>
     </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
       <c r="D124" s="1"/>
@@ -2441,7 +2449,7 @@
       <c r="F124" s="1"/>
       <c r="G124" s="1"/>
     </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
       <c r="D125" s="1"/>
@@ -2449,7 +2457,7 @@
       <c r="F125" s="1"/>
       <c r="G125" s="1"/>
     </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
       <c r="D126" s="1"/>
@@ -2457,7 +2465,7 @@
       <c r="F126" s="1"/>
       <c r="G126" s="1"/>
     </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
       <c r="D127" s="1"/>
@@ -2465,7 +2473,7 @@
       <c r="F127" s="1"/>
       <c r="G127" s="1"/>
     </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
       <c r="D128" s="1"/>
@@ -2473,7 +2481,7 @@
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
     </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
       <c r="D129" s="1"/>
@@ -2481,7 +2489,7 @@
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
     </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
       <c r="D130" s="1"/>
@@ -2489,7 +2497,7 @@
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
     </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
       <c r="D131" s="1"/>
@@ -2497,7 +2505,7 @@
       <c r="F131" s="1"/>
       <c r="G131" s="1"/>
     </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
       <c r="D132" s="1"/>
@@ -2505,7 +2513,7 @@
       <c r="F132" s="1"/>
       <c r="G132" s="1"/>
     </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
       <c r="D133" s="1"/>
@@ -2513,7 +2521,7 @@
       <c r="F133" s="1"/>
       <c r="G133" s="1"/>
     </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
       <c r="D134" s="1"/>
@@ -2521,7 +2529,7 @@
       <c r="F134" s="1"/>
       <c r="G134" s="1"/>
     </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
       <c r="D135" s="1"/>
@@ -2529,7 +2537,7 @@
       <c r="F135" s="1"/>
       <c r="G135" s="1"/>
     </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
       <c r="D136" s="1"/>
@@ -2537,7 +2545,7 @@
       <c r="F136" s="1"/>
       <c r="G136" s="1"/>
     </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
       <c r="D137" s="1"/>
@@ -2545,7 +2553,7 @@
       <c r="F137" s="1"/>
       <c r="G137" s="1"/>
     </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
       <c r="D138" s="1"/>
@@ -2553,7 +2561,7 @@
       <c r="F138" s="1"/>
       <c r="G138" s="1"/>
     </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
       <c r="D139" s="1"/>
@@ -2561,7 +2569,7 @@
       <c r="F139" s="1"/>
       <c r="G139" s="1"/>
     </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
       <c r="D140" s="1"/>
@@ -2569,7 +2577,7 @@
       <c r="F140" s="1"/>
       <c r="G140" s="1"/>
     </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
       <c r="D141" s="1"/>
@@ -2577,7 +2585,7 @@
       <c r="F141" s="1"/>
       <c r="G141" s="1"/>
     </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
       <c r="D142" s="1"/>
@@ -2585,7 +2593,7 @@
       <c r="F142" s="1"/>
       <c r="G142" s="1"/>
     </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
       <c r="D143" s="1"/>
@@ -2593,7 +2601,7 @@
       <c r="F143" s="1"/>
       <c r="G143" s="1"/>
     </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
       <c r="D144" s="1"/>
@@ -2601,7 +2609,7 @@
       <c r="F144" s="1"/>
       <c r="G144" s="1"/>
     </row>
-    <row r="145" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
       <c r="D145" s="1"/>
@@ -2609,7 +2617,7 @@
       <c r="F145" s="1"/>
       <c r="G145" s="1"/>
     </row>
-    <row r="146" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
       <c r="D146" s="1"/>
@@ -2617,7 +2625,7 @@
       <c r="F146" s="1"/>
       <c r="G146" s="1"/>
     </row>
-    <row r="147" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
       <c r="D147" s="1"/>
@@ -2625,7 +2633,7 @@
       <c r="F147" s="1"/>
       <c r="G147" s="1"/>
     </row>
-    <row r="148" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
       <c r="D148" s="1"/>
@@ -2633,7 +2641,7 @@
       <c r="F148" s="1"/>
       <c r="G148" s="1"/>
     </row>
-    <row r="149" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
       <c r="D149" s="1"/>
@@ -2641,29 +2649,21 @@
       <c r="F149" s="1"/>
       <c r="G149" s="1"/>
     </row>
-    <row r="150" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B150" s="1"/>
-      <c r="C150" s="1"/>
-      <c r="D150" s="1"/>
-      <c r="E150" s="1"/>
-      <c r="F150" s="1"/>
-      <c r="G150" s="1"/>
-    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A35:A41"/>
-    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="A34:A40"/>
+    <mergeCell ref="A24:A28"/>
     <mergeCell ref="A5:A8"/>
-    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A29:A33"/>
     <mergeCell ref="A9:A16"/>
-    <mergeCell ref="A17:A24"/>
+    <mergeCell ref="A17:A23"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B150" xr:uid="{E9C7F5BF-2317-44E3-A3AA-39649CD07628}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B149" xr:uid="{E9C7F5BF-2317-44E3-A3AA-39649CD07628}">
       <formula1>"GET, PUT, POST, PATCH, DELETE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H41" xr:uid="{8B853124-466D-458F-830D-86556B38ED3C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H40" xr:uid="{8B853124-466D-458F-830D-86556B38ED3C}">
       <formula1>"Not done, Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>